<commit_message>
imports correctly and asdownload uses args when not run interactively
</commit_message>
<xml_diff>
--- a/asInventory.xlsx
+++ b/asInventory.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gw234478\win\asInventory\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gw234478\projects\asInventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9365123C-394B-476E-8FBC-6B04F5B2C3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21210" windowHeight="7590"/>
+    <workbookView xWindow="-28800" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -19,15 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Title</t>
-  </si>
-  <si>
-    <t>Level</t>
-  </si>
-  <si>
-    <t>Ref ID</t>
   </si>
   <si>
     <t>ID</t>
@@ -99,8 +94,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,25 +103,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -138,16 +121,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Accent1" xfId="1" builtinId="29"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -175,7 +155,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -192,32 +172,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Inventory" displayName="Inventory" ref="A6:W13">
-  <autoFilter ref="A6:W13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Inventory" displayName="Inventory" ref="A1:W8">
+  <autoFilter ref="A1:W8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="23">
-    <tableColumn id="1" name="ID"/>
-    <tableColumn id="2" name="Location ID"/>
-    <tableColumn id="3" name="Location"/>
-    <tableColumn id="4" name="Container URI"/>
-    <tableColumn id="5" name="Container"/>
-    <tableColumn id="6" name="C#"/>
-    <tableColumn id="7" name="Folder"/>
-    <tableColumn id="8" name="F#"/>
-    <tableColumn id="9" name="Title"/>
-    <tableColumn id="10" name="Date 1 Display"/>
-    <tableColumn id="11" name="Date 1 Normal"/>
-    <tableColumn id="12" name="Date 2 Display"/>
-    <tableColumn id="13" name="Date 2 Normal"/>
-    <tableColumn id="14" name="Date 3 Display"/>
-    <tableColumn id="15" name="Date 3 Normal"/>
-    <tableColumn id="16" name="Date 4 Display"/>
-    <tableColumn id="17" name="Date 4 Normal"/>
-    <tableColumn id="18" name="Date 5 Display"/>
-    <tableColumn id="19" name="Date 5 Normal"/>
-    <tableColumn id="20" name="Restrictions"/>
-    <tableColumn id="21" name="General Note"/>
-    <tableColumn id="22" name="Scope"/>
-    <tableColumn id="23" name="DAO Filename"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Location ID"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Location"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Container URI"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Container"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="C#"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Folder"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="F#"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Title"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Date 1 Display"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Date 1 Normal"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Date 2 Display"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Date 2 Normal"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Date 3 Display"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Date 3 Normal"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Date 4 Display"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Date 4 Normal"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Date 5 Display"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Date 5 Normal"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Restrictions"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="General Note"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Scope"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="DAO Filename"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -507,8 +487,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:W1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="15" customWidth="1"/>
@@ -516,90 +496,75 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H1" s="1" t="s">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="H6" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="I6" t="s">
-        <v>0</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="K6" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="L6" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="M6" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="N6" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="P6" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="R6" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="S6" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="T6" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="U6" t="s">
+      <c r="W1" t="s">
         <v>22</v>
-      </c>
-      <c r="V6" t="s">
-        <v>23</v>
-      </c>
-      <c r="W6" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>